<commit_message>
feat: draw Excel routes and add map distance measurement
</commit_message>
<xml_diff>
--- a/sample_map_data.xlsx
+++ b/sample_map_data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="markers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lines" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="polygons" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="heatmap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="circles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="markers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="lines" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="polygons" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="heatmap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="circles" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -352,7 +352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="2" min="1" max="1"/>
@@ -532,6 +532,62 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>orange</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>25.7984</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-80.20269999999999</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CMU Miami</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University Miami campus</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>25.795</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-80.2867</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Miami International Airport</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Miami International Airport (MIA)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>plane</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>blue</t>
         </is>
       </c>
     </row>
@@ -548,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="2" min="1" max="1"/>
@@ -629,6 +685,29 @@
       </c>
       <c r="E3" s="2" t="n">
         <v>0.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CMU Miami to MIA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[[25.7984, -80.2027], [25.795, -80.2867]]</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>